<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-01 La tour de cubes
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-01.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-01.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison</t>
+          <t>maison, salon, cubes, carton, bois, fenêtre, soleil, peinture, sol</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, papa</t>
+          <t>Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël construit une tour. Les cubes tombent. Il est surpris. Il souffle, s'assoit, fait une pause. Puis il reprend, tout doucement.</t>
+          <t>Le bois des cubes sent le soleil. Sur le bois, un éclat de tour luit. Mila veut empiler, maintenant. Les cubes tombent. Poitrine trop vite. Sourire parti. Papa s'accroupit. Elle souffle, pause. Merci vécu. Deuxième ruse : trop de cubes, la tour penche. Elle refuse de foncer. Un éclat de tour tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La pluie vient de s'arrêter. Des gouttes brillent à la fenêtre. Elles ressemblent à des perles. Le tapis beige est épais. Les pantoufles de papa glissent tout bas. Tu as vu les gouttes, Raphaël ? Oui, papa. Ça brille. La pluie a fini. Une tour de cubes rouges attend. Les cubes sont lisses et froids. En ce moment, Raphaël construit. Il pose un cube. Puis un autre. La tour monte. Les cubes tombent. Ça fait du bruit. Raphaël est surpris. Les cubes sont tombés d'un coup. Sa poitrine va trop vite. Ses mains tremblent un peu. C'est trop. On peut souffler. Papa est sur le tapis. Souffle comme le vent. Raphaël souffle comme le vent. Une fois. Deux fois. Il s'assoit. Il fait une pause. Ses mains se posent sur ses genoux. Bravo, Raphaël. Tu as soufflé. Tu as fait une pause. Ton corps va plus doucement, maintenant ? Oui, papa. Le salon redevient calme. Raphaël reprend un cube. Il construit tout doucement. On reprend, tout doucement. Papa reste près de lui. Souffler, puis une pause. On peut reprendre. Un cube rouge tapote le tapis. Raphaël le pose tout doucement. La tour a deux cubes. Elle tient, cette fois. Tu as pris ton temps. Elle tient, papa. Les gouttes glissent sur la vitre. Elles font un petit chemin. On regarde les gouttes un moment ? Oui.</t>
+          <t>Le bois des cubes sent le soleil. Ça sent le bois, papa. Tu le sens, le bois chaud ? Oui, papa. Un cube tape un autre cube. Toc, près de la fenêtre. Tu entends le toc, Mila ? Oui, maman. La peinture des cubes est un peu collante. Elle colle aux doigts. Elle est tiède, Mila ? Un peu, maman. Papa ouvre le carton des cubes. Le carton froisse, près des genoux. Tu vois les cubes, Mila ? Oui, ils brillent. Un cube jaune roule vers le sol. Il est jaune ! Tu le rattrapes ? Oui, maman. Sur le bois, un éclat de tour luit. Il brille, maman. Tu le vois, sur le bois ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. La fenêtre chauffe le salon. Elle est chaude. Tu poses un cube, Mila ? Oui. Maman s'assoit près du carton. Ça chauffe les genoux. Les genoux sont bien ? Oui, papa. Un cube bleu attend dans la main. Il est lisse. Il sent la peinture ? Un peu, maman. En ce moment, Mila prend un cube. Je veux empiler, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le bois peint. Tu mets le cube dessus ? Oui, maman. Mila pose un cube trop vite. Puis un autre, trop haut. Plus haut ! La tour penche d'un coup. Les cubes tombent sur le sol. Ça fait un bruit sec. Oh. Mila reste surprise, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Mila ? Oui, papa. Tes mains sont chaudes, Mila ? Un peu, maman. L'éclat de tour tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La pluie vient de s'arrêter. Des gouttes brillent à la fenêtre. Elles ressemblent à des perles. Le tapis beige est épais. Les pantoufles de papa glissent tout bas. Tu as vu les gouttes, Raphaël ? Oui, papa. Ça brille. La pluie a fini. Une tour de cubes rouges attend. Les cubes sont lisses et froids. En ce moment, Raphaël construit. Il pose un cube. Puis un autre. La tour monte. Les cubes tombent. Ça fait du bruit. Raphaël est surpris. Les cubes sont tombés d'un coup. Sa poitrine va trop vite. Ses mains tremblent un peu. C'est trop. On peut souffler. Papa est sur le tapis. Souffle comme le vent. Raphaël souffle comme le vent. Une fois. Deux fois. Il s'assoit. Il fait une pause. Ses mains se posent sur ses genoux. Bravo, Raphaël. Tu as soufflé. Tu as fait une pause. Ton corps va plus doucement, maintenant ? Oui, papa. Le salon redevient calme. Raphaël reprend un cube. Il construit tout doucement. On reprend, tout doucement. Papa reste près de lui. Souffler, puis une pause. On peut reprendre. Un cube rouge tapote le tapis. Raphaël le pose tout doucement. La tour a deux cubes. Elle tient, cette fois. Tu as pris ton temps. Elle tient, papa. Les gouttes glissent sur la vitre. Elles font un petit chemin. On regarde les gouttes un moment ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le bois des cubes sent le soleil. Ça sent le bois, papa. Tu le sens, le bois chaud ? Oui, papa. Un cube tape un autre cube. Toc, près de la fenêtre. Tu entends le toc, Mila ? Oui, maman. La peinture des cubes est un peu collante. Elle colle aux doigts. Elle est tiède, Mila ? Un peu, maman. Papa ouvre le carton des cubes. Le carton froisse, près des genoux. Tu vois les cubes, Mila ? Oui, ils brillent. Un cube jaune roule vers le sol. Il est jaune ! Tu le rattrapes ? Oui, maman. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de tour&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bois ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. La fenêtre chauffe le salon. Elle est chaude. Tu poses un cube, Mila ? Oui. Maman s'assoit près du carton. Ça chauffe les genoux. Les genoux sont bien ? Oui, papa. Un cube bleu attend dans la main. Il est lisse. Il sent la peinture ? Un peu, maman. En ce moment, Mila prend un cube. Je veux empiler, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le bois peint. Tu mets le cube dessus ? Oui, maman. Mila pose un cube trop vite. Puis un autre, trop haut. Plus haut ! La tour penche d'un coup. Les cubes tombent sur le sol. Ça fait un bruit sec. Oh. Mila reste surprise, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Mila ? Oui, papa. Tes mains sont chaudes, Mila ? Un peu, maman. L'éclat de tour tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila joue dans le salon. Les cubes tombent. Ça fait du bruit. Lila sent sa poitrine aller vite. Elle dit : c'est trop. Papa est là, sur le tapis. Papa dit : on peut &lt;emphasis&gt;souffler&lt;/emphasis&gt;. Lila souffle comme le vent. Une fois. Deux fois. Elle s'assoit. Elle fait une pause. Ses mains se posent sur ses genoux. Le salon redevient calme. Lila reprend un cube. Elle construit tout doucement. Papa reste près d'elle. Souffler, puis une pause. On peut reprendre.&lt;/slow&gt; [pause]</t>
+          <t>Le bois des cubes sent le soleil. Ça sent le bois, papa. Tu le sens, le bois chaud ? Oui, papa. Un cube tape un autre cube. Toc, près de la fenêtre. Tu entends le toc, Mila ? Oui, maman. La peinture des cubes est un peu collante. Elle colle aux doigts. Elle est tiède, Mila ? Un peu, maman. Papa ouvre le carton des cubes. Le carton froisse, près des genoux. Tu vois les cubes, Mila ? Oui, ils brillent. Un cube jaune roule vers le sol. Il est jaune ! Tu le rattrapes ? Oui, maman. Sur le bois, un &lt;emphasis&gt;éclat de tour&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bois ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. La fenêtre chauffe le salon. Elle est chaude. Tu poses un cube, Mila ? Oui. Maman s'assoit près du carton. Ça chauffe les genoux. Les genoux sont bien ? Oui, papa. Un cube bleu attend dans la main. Il est lisse. Il sent la peinture ? Un peu, maman. En ce moment, Mila prend un cube. Je veux empiler, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le bois peint. Tu mets le cube dessus ? Oui, maman. Mila pose un cube trop vite. Puis un autre, trop haut. Plus haut ! La tour penche d'un coup. Les cubes tombent sur le sol. Ça fait un bruit sec. Oh. Mila reste surprise, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Mila ? Oui, papa. Tes mains sont chaudes, Mila ? Un peu, maman. L'éclat de tour tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>souffler</t>
+          <t>éclat de tour</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,63 +1324,79 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_empiler_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La pluie vient de s'arrêter.
-narrateur|Des gouttes brillent à la fenêtre.
-narrateur|Elles ressemblent à des perles.
-narrateur|Le tapis beige est épais.
-narrateur|Les pantoufles de papa glissent tout bas.
-papa|Tu as vu les gouttes, Raphaël ?
-enfant-m|Oui, papa. Ça brille.
-papa|La pluie a fini.
-narrateur|Une tour de cubes rouges attend.
-narrateur|Les cubes sont lisses et froids.
-narrateur|En ce moment, Raphaël construit.
-narrateur|Il pose un cube.
-narrateur|Puis un autre.
-narrateur|La tour monte.
-narrateur|Les cubes tombent.
-narrateur|Ça fait du bruit.
-narrateur|Raphaël est surpris.
-narrateur|Les cubes sont tombés d'un coup.
+          <t>narrateur|Le bois des cubes sent le soleil.
+enfant-f|Ça sent le bois, papa.
+papa|Tu le sens, le bois chaud ?
+enfant-f|Oui, papa.
+narrateur|Un cube tape un autre cube.
+narrateur|Toc, près de la fenêtre.
+maman|Tu entends le toc, Mila ?
+enfant-f|Oui, maman.
+narrateur|La peinture des cubes est un peu collante.
+enfant-f|Elle colle aux doigts.
+maman|Elle est tiède, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Papa ouvre le carton des cubes.
+narrateur|Le carton froisse, près des genoux.
+papa|Tu vois les cubes, Mila ?
+enfant-f|Oui, ils brillent.
+narrateur|Un cube jaune roule vers le sol.
+enfant-f|Il est jaune !
+maman|Tu le rattrapes ?
+enfant-f|Oui, maman.
+narrateur|Sur le bois, un éclat de tour luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, sur le bois ?
+enfant-f|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse sur le bord.
+narrateur|La fenêtre chauffe le salon.
+enfant-f|Elle est chaude.
+maman|Tu poses un cube, Mila ?
+enfant-f|Oui.
+narrateur|Maman s'assoit près du carton.
+enfant-f|Ça chauffe les genoux.
+papa|Les genoux sont bien ?
+enfant-f|Oui, papa.
+narrateur|Un cube bleu attend dans la main.
+enfant-f|Il est lisse.
+maman|Il sent la peinture ?
+enfant-f|Un peu, maman.
+narrateur|En ce moment, Mila prend un cube.
+enfant-f|Je veux empiler, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Les mains serrent le bois peint.
+maman|Tu mets le cube dessus ?
+enfant-f|Oui, maman.
+narrateur|Mila pose un cube trop vite.
+narrateur|Puis un autre, trop haut.
+enfant-f|Plus haut !
+narrateur|La tour penche d'un coup.
+narrateur|Les cubes tombent sur le sol.
+narrateur|Ça fait un bruit sec.
+enfant-f|Oh.
+narrateur|Mila reste surprise, les mains ouvertes.
 narrateur|Sa poitrine va trop vite.
-narrateur|Ses mains tremblent un peu.
-enfant-m|C'est trop.
-papa|On peut souffler.
-narrateur|Papa est sur le tapis.
-papa|Souffle comme le vent.
-narrateur|Raphaël souffle comme le vent.
-narrateur|Une fois.
-narrateur|Deux fois.
-narrateur|Il s'assoit.
-narrateur|Il fait une pause.
-narrateur|Ses mains se posent sur ses genoux.
-papa|Bravo, Raphaël.
-papa|Tu as soufflé.
-papa|Tu as fait une pause.
-papa|Ton corps va plus doucement, maintenant ?
-enfant-m|Oui, papa.
-narrateur|Le salon redevient calme.
-narrateur|Raphaël reprend un cube.
-narrateur|Il construit tout doucement.
-papa|On reprend, tout doucement.
-narrateur|Papa reste près de lui.
-narrateur|Souffler, puis une pause.
-narrateur|On peut reprendre.
-narrateur|Un cube rouge tapote le tapis.
-narrateur|Raphaël le pose tout doucement.
-narrateur|La tour a deux cubes.
-papa|Elle tient, cette fois.
-papa|Tu as pris ton temps.
-enfant-m|Elle tient, papa.
-narrateur|Les gouttes glissent sur la vitre.
-narrateur|Elles font un petit chemin.
-papa|On regarde les gouttes un moment ?
-enfant-m|Oui.</t>
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois les cubes, Mila ?
+enfant-f|Oui, papa.
+maman|Tes mains sont chaudes, Mila ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de tour tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1412,17 +1428,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Raphaël va vite. Que fait-il ?</t>
+          <t>Le corps de Mila va vite. Que fait-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Raphaël va vite. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le corps de &lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt; va vite. Que fait-elle ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le corps de Lila va vite. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le corps de &lt;emphasis&gt;Mila&lt;/emphasis&gt; va vite. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1447,7 +1463,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Papa dit de souffler. Que fait Lila ensuite ?</t>
+          <t>Papa dit de souffler. Que fait Mila ensuite ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1485,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1496,7 +1512,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1511,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1553,7 +1573,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1563,12 +1583,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_corps_de_mila_va_vite_que_fait_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Le corps de Raphaël va vite. Que fait-il ?</t>
+          <t>narrateur|Le corps de Mila va vite.
+narrateur|Que fait-elle ?</t>
         </is>
       </c>
     </row>
@@ -1595,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a soufflé. Il a fait une pause. Son corps a ralenti. Tu as soufflé comme le vent. Bravo. Tu restes assis un peu ? Oui. Les cubes rouges attendent. Les gouttes brillent encore.</t>
+          <t>Mila veut empiler, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre. Les mots se bousculent dans sa bouche. Trop vite. Mila avance les mains, trop vite. Puis elle s'arrête. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les cubes, un instant. Elle écoute le salon. Pouh. Mila souffle une fois. Elle souffle une deuxième fois. Elle s'assoit près du carton. Ses mains se posent sur ses genoux. La poitrine ralentit un peu. Tu restes un peu, Mila ? Oui, papa. Merci, Mila. Papa reste à la même hauteur. La peinture colle un peu, sous les doigts. Elle est tiède. Mila reprend un cube, sans se presser. Elle le pose sur un autre. Tu le vois, le cube ? Oui, papa. Il tient, Mila ? Oui, maman. La tour a deux cubes. Elle tient ! La tour est calme ? Oui, papa. Tes mains sont au chaud ? Un peu, maman. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Le rayon touche le bord ? Oui, maman. Le cube jaune attend à côté. Je le prends. Tu le poses, Mila ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a soufflé. Il a fait une pause. Son corps a ralenti. Tu as soufflé comme le vent. Bravo. Tu restes assis un peu ? Oui. Les cubes rouges attendent. Les gouttes brillent encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut empiler, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre. Les mots se bousculent dans sa bouche. Trop vite. Mila avance les mains, trop vite. Puis elle s'arrête. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les cubes, un instant. Elle écoute le salon. Pouh. Mila &lt;emphasis level="moderate"&gt;souffle&lt;/emphasis&gt; une fois. Elle souffle une deuxième fois. Elle s'assoit près du carton. Ses mains se posent sur ses genoux. La poitrine ralentit un peu. Tu restes un peu, Mila ? Oui, papa. Merci, Mila. Papa reste à la même hauteur. La peinture colle un peu, sous les doigts. Elle est tiède. Mila reprend un cube, sans se presser. Elle le pose sur un autre. Tu le vois, le cube ? Oui, papa. Il tient, Mila ? Oui, maman. La tour a deux cubes. Elle tient ! La tour est calme ? Oui, papa. Tes mains sont au chaud ? Un peu, maman. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Le rayon touche le bord ? Oui, maman. Le cube jaune attend à côté. Je le prends. Tu le poses, Mila ? Oui, papa.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila a soufflé. Elle a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Son corps a ralenti.&lt;/slow&gt; [pause]</t>
+          <t>Mila veut empiler, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre. Les mots se bousculent dans sa bouche. Trop vite. Mila avance les mains, trop vite. Puis elle s'arrête. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les cubes, un instant. Elle écoute le salon. Pouh. Mila &lt;emphasis&gt;souffle&lt;/emphasis&gt; une fois. Elle souffle une deuxième fois. Elle s'assoit près du carton. Ses mains se posent sur ses genoux. La poitrine ralentit un peu. Tu restes un peu, Mila ? Oui, papa. Merci, Mila. Papa reste à la même hauteur. La peinture colle un peu, sous les doigts. Elle est tiède. Mila reprend un cube, sans se presser. Elle le pose sur un autre. Tu le vois, le cube ? Oui, papa. Il tient, Mila ? Oui, maman. La tour a deux cubes. Elle tient ! La tour est calme ? Oui, papa. Tes mains sont au chaud ? Un peu, maman. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Le rayon touche le bord ? Oui, maman. Le cube jaune attend à côté. Je le prends. Tu le poses, Mila ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1652,18 +1673,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1686,30 +1707,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>souffle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1718,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1730,24 +1751,61 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_souffle_elle_fait_une_pause; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a soufflé.
-narrateur|Il a fait une pause.
-narrateur|Son corps a ralenti.
-papa|Tu as soufflé comme le vent.
-papa|Bravo.
-papa|Tu restes assis un peu ?
-enfant-m|Oui.
-narrateur|Les cubes rouges attendent.
-narrateur|Les gouttes brillent encore.</t>
+          <t>narrateur|Mila veut empiler, tout de suite.
+enfant-f|Je mets tout, maintenant !
+narrateur|Les cubes restent par terre.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Trop vite.
+narrateur|Mila avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe les cubes, un instant.
+narrateur|Elle écoute le salon.
+enfant-f|Pouh.
+narrateur|Mila souffle une fois.
+narrateur|Elle souffle une deuxième fois.
+narrateur|Elle s'assoit près du carton.
+narrateur|Ses mains se posent sur ses genoux.
+narrateur|La poitrine ralentit un peu.
+papa|Tu restes un peu, Mila ?
+enfant-f|Oui, papa.
+papa|Merci, Mila.
+narrateur|Papa reste à la même hauteur.
+maman|La peinture colle un peu, sous les doigts.
+enfant-f|Elle est tiède.
+narrateur|Mila reprend un cube, sans se presser.
+narrateur|Elle le pose sur un autre.
+papa|Tu le vois, le cube ?
+enfant-f|Oui, papa.
+maman|Il tient, Mila ?
+enfant-f|Oui, maman.
+narrateur|La tour a deux cubes.
+enfant-f|Elle tient !
+papa|La tour est calme ?
+enfant-f|Oui, papa.
+maman|Tes mains sont au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près des cubes ?
+enfant-f|Oui.
+maman|Le rayon touche le bord ?
+enfant-f|Oui, maman.
+narrateur|Le cube jaune attend à côté.
+enfant-f|Je le prends.
+papa|Tu le poses, Mila ?
+enfant-f|Oui, papa.</t>
         </is>
       </c>
     </row>
@@ -1774,17 +1832,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël pose un cube rouge. Papa reste sur le tapis. La tour recommence. Tout doucement. Tu veux encore souffler une fois ? Oui. Raphaël souffle. Il fait encore une petite pause. Puis il pose un autre cube. La tour a trois cubes. Elle ne tombe pas. Tu as pris le temps. Bravo.</t>
+          <t>Maman pousse le carton près du sol. Il est un peu poudreux. La tour, maintenant ! Mila prend trop de cubes, tout de suite. Un cube glisse de sa main. Il glisse ! La tour penche vers le carton. Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la tour, un instant. Elle écoute le salon, près des cubes. Sur le bois, un éclat de tour luit. Là, sur le bois. Mila souffle une fois. Elle attend, assise un moment. Pouh. On tient le cube ? Oui, papa. Le cube sent le bois chaud. La tour est là, un peu penchée. Mila pose le cube, sans se presser. La tour se redresse. Poumf. Le bois est tiède, Mila ? Un peu. Elle pose un autre cube, au milieu. La tour est bien calme ? Oui, papa. Un rayon passe sur le bord. Il allume le bois. Tu vois le point, Mila ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. La tour est calme ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le carton reste ouvert, près d'elle. Il sent le bois. On reste ici, Mila ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël pose un cube rouge. Papa reste sur le tapis. La tour recommence. Tout doucement. Tu veux encore souffler une fois ? Oui. Raphaël souffle. Il fait encore une petite pause. Puis il pose un autre cube. La tour a trois cubes. Elle ne tombe pas. Tu as pris le temps. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse le carton près du sol. Il est un peu poudreux. La tour, maintenant ! Mila prend trop de cubes, tout de suite. Un cube glisse de sa main. Il glisse ! La tour penche vers le carton. Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la tour, un instant. Elle écoute le salon, près des cubes. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de tour&lt;/emphasis&gt; luit. Là, sur le bois. Mila souffle une fois. Elle attend, assise un moment. Pouh. On tient le cube ? Oui, papa. Le cube sent le bois chaud. La tour est là, un peu penchée. Mila pose le cube, sans se presser. La tour se redresse. Poumf. Le bois est tiède, Mila ? Un peu. Elle pose un autre cube, au milieu. La tour est bien calme ? Oui, papa. Un rayon passe sur le bord. Il allume le bois. Tu vois le point, Mila ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. La tour est calme ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le carton reste ouvert, près d'elle. Il sent le bois. On reste ici, Mila ? Oui.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila pose un cube rouge. Papa reste sur le tapis.&lt;/slow&gt; [pause]</t>
+          <t>Maman pousse le carton près du sol. Il est un peu poudreux. La tour, maintenant ! Mila prend trop de cubes, tout de suite. Un cube glisse de sa main. Il glisse ! La tour penche vers le carton. Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la tour, un instant. Elle écoute le salon, près des cubes. Sur le bois, un &lt;emphasis&gt;éclat de tour&lt;/emphasis&gt; luit. Là, sur le bois. Mila souffle une fois. Elle attend, assise un moment. Pouh. On tient le cube ? Oui, papa. Le cube sent le bois chaud. La tour est là, un peu penchée. Mila pose le cube, sans se presser. La tour se redresse. Poumf. Le bois est tiède, Mila ? Un peu. Elle pose un autre cube, au milieu. La tour est bien calme ? Oui, papa. Un rayon passe sur le bord. Il allume le bois. Tu vois le point, Mila ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. La tour est calme ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le carton reste ouvert, près d'elle. Il sent le bois. On reste ici, Mila ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1831,18 +1889,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1863,28 +1921,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tour</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1893,10 +1955,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1905,24 +1967,60 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=trop_de_cubes_la_tour_penche_elle_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël pose un cube rouge.
-narrateur|Papa reste sur le tapis.
-papa|La tour recommence.
-papa|Tout doucement.
-papa|Tu veux encore souffler une fois ?
-enfant-m|Oui.
-narrateur|Raphaël souffle.
-narrateur|Il fait encore une petite pause.
-narrateur|Puis il pose un autre cube.
-narrateur|La tour a trois cubes.
-narrateur|Elle ne tombe pas.
-papa|Tu as pris le temps.
-papa|Bravo.</t>
+          <t>narrateur|Maman pousse le carton près du sol.
+narrateur|Il est un peu poudreux.
+enfant-f|La tour, maintenant !
+narrateur|Mila prend trop de cubes, tout de suite.
+narrateur|Un cube glisse de sa main.
+enfant-f|Il glisse !
+narrateur|La tour penche vers le carton.
+narrateur|Mila avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la tour, un instant.
+narrateur|Elle écoute le salon, près des cubes.
+narrateur|Sur le bois, un éclat de tour luit.
+enfant-f|Là, sur le bois.
+narrateur|Mila souffle une fois.
+narrateur|Elle attend, assise un moment.
+enfant-f|Pouh.
+papa|On tient le cube ?
+enfant-f|Oui, papa.
+narrateur|Le cube sent le bois chaud.
+narrateur|La tour est là, un peu penchée.
+narrateur|Mila pose le cube, sans se presser.
+narrateur|La tour se redresse.
+enfant-f|Poumf.
+maman|Le bois est tiède, Mila ?
+enfant-f|Un peu.
+narrateur|Elle pose un autre cube, au milieu.
+papa|La tour est bien calme ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le bord.
+enfant-f|Il allume le bois.
+papa|Tu vois le point, Mila ?
+enfant-f|Oui, papa.
+narrateur|Les cubes tiennent, l'un sur l'autre.
+enfant-f|C'est plus facile.
+papa|La tour est calme ?
+enfant-f|Oui, papa.
+maman|Tes genoux sont au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Le carton reste ouvert, près d'elle.
+enfant-f|Il sent le bois.
+papa|On reste ici, Mila ?
+enfant-f|Oui.</t>
         </is>
       </c>
     </row>
@@ -1949,17 +2047,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo. On a repris, tout doucement.</t>
+          <t>Ils restent près du carton. Maman essuie un peu de peinture. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près de la tour. On est bien, ici. Mila tapote le bois du doigt. Il a une trace de peinture. Tu la vois, la trace ? Oui, maman. La tour est restée, Mila. Oui, avec les cubes. Ça sent le bois, un peu tiède. Et la peinture, maman. Oui, dans l'air. Le salon est calme, Mila ? Oui, papa. La tour reste près du carton. Un éclat de tour tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo. On a repris, tout doucement.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du carton. Maman essuie un peu de peinture. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près de la tour. On est bien, ici. Mila tapote le bois du doigt. Il a une trace de peinture. Tu la vois, la trace ? Oui, maman. La tour est restée, Mila. Oui, avec les cubes. Ça sent le bois, un peu tiède. Et la peinture, maman. Oui, dans l'air. Le salon est calme, Mila ? Oui, papa. La tour reste près du carton. Un &lt;emphasis level="moderate"&gt;éclat de tour&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du carton. Maman essuie un peu de peinture. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près de la tour. On est bien, ici. Mila tapote le bois du doigt. Il a une trace de peinture. Tu la vois, la trace ? Oui, maman. La tour est restée, Mila. Oui, avec les cubes. Ça sent le bois, un peu tiède. Et la peinture, maman. Oui, dans l'air. Le salon est calme, Mila ? Oui, papa. La tour reste près du carton. Un &lt;emphasis&gt;éclat de tour&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2006,7 +2104,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2014,7 +2112,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2026,12 +2124,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2040,14 +2138,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tour</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2059,11 +2161,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2072,27 +2174,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai soufflé.
-enfant-m|J'ai fait une pause.
-papa|Bravo.
-papa|On a repris, tout doucement.</t>
+          <t>narrateur|Ils restent près du carton.
+narrateur|Maman essuie un peu de peinture.
+enfant-f|Les cubes sont tombés, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, près de la tour.
+maman|On est bien, ici.
+narrateur|Mila tapote le bois du doigt.
+enfant-f|Il a une trace de peinture.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|La tour est restée, Mila.
+enfant-f|Oui, avec les cubes.
+narrateur|Ça sent le bois, un peu tiède.
+enfant-f|Et la peinture, maman.
+maman|Oui, dans l'air.
+papa|Le salon est calme, Mila ?
+enfant-f|Oui, papa.
+narrateur|La tour reste près du carton.
+narrateur|Un éclat de tour tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2170,6 +2291,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>